<commit_message>
feat: add blank templates (for download) + real-data templates (for testing)
- bachelor_upload_template.xlsx / master_upload_template.xlsx — blank with example row (for user download)
- bachelor_upload_template_with_data.xlsx / master_upload_template_with_data.xlsx — populated with real DB students (for testing)
- Updated generate-samples.js to create both versions
- Frontend public/ gets blank templates for download
</commit_message>
<xml_diff>
--- a/backend/excel-templates/bachelor_upload_template.xlsx
+++ b/backend/excel-templates/bachelor_upload_template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -418,19 +418,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>SampleGroup1</v>
+        <v/>
       </c>
       <c r="B2" t="str">
-        <v>Sample Bachelor Project 1</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>Aarav Khadka</v>
+        <v/>
       </c>
       <c r="D2" t="str">
-        <v>078BCT001</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v>2081</v>
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -441,137 +441,18 @@
         <v>Sample Bachelor Project 1</v>
       </c>
       <c r="C3" t="str">
-        <v>Binita Shrestha</v>
+        <v>Aarav Khadka, Binita Shrestha, Chandra Thapa</v>
       </c>
       <c r="D3" t="str">
-        <v>078BCT002</v>
+        <v>078BCT001, 078BCT002, 078BCT003</v>
       </c>
       <c r="E3" t="str">
-        <v>2081</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>SampleGroup1</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Sample Bachelor Project 1</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Chandra Thapa</v>
-      </c>
-      <c r="D4" t="str">
-        <v>078BCT003</v>
-      </c>
-      <c r="E4" t="str">
-        <v>2081</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>SampleGroup2</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Sample Bachelor Project 2</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Deepa Poudel</v>
-      </c>
-      <c r="D5" t="str">
-        <v>078BCT004</v>
-      </c>
-      <c r="E5" t="str">
-        <v>2081</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>SampleGroup2</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Sample Bachelor Project 2</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Ekaraj Rana</v>
-      </c>
-      <c r="D6" t="str">
-        <v>078BCT005</v>
-      </c>
-      <c r="E6" t="str">
-        <v>2081</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>SampleGroup2</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Sample Bachelor Project 2</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Falguni Neupane</v>
-      </c>
-      <c r="D7" t="str">
-        <v>078BCT006</v>
-      </c>
-      <c r="E7" t="str">
-        <v>2081</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>SampleGroup3</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Sample Bachelor Project 3</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Ganesh Bhandari</v>
-      </c>
-      <c r="D8" t="str">
-        <v>078BCT007</v>
-      </c>
-      <c r="E8" t="str">
-        <v>2081</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>SampleGroup3</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Sample Bachelor Project 3</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Hima Acharya</v>
-      </c>
-      <c r="D9" t="str">
-        <v>078BCT008</v>
-      </c>
-      <c r="E9" t="str">
-        <v>2081</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>SampleGroup3</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Sample Bachelor Project 3</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Indra Joshi</v>
-      </c>
-      <c r="D10" t="str">
-        <v>078BCT009</v>
-      </c>
-      <c r="E10" t="str">
         <v>2081</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Applied all requested changes
</commit_message>
<xml_diff>
--- a/backend/excel-templates/bachelor_upload_template.xlsx
+++ b/backend/excel-templates/bachelor_upload_template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:G4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,6 +415,12 @@
       <c r="E1" t="str">
         <v>Academic Year</v>
       </c>
+      <c r="F1" t="str">
+        <v>Supervisor</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Examiner</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -432,13 +438,19 @@
       <c r="E2" t="str">
         <v/>
       </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>SampleGroup1</v>
+        <v>TeamAlpha</v>
       </c>
       <c r="B3" t="str">
-        <v>Sample Bachelor Project 1</v>
+        <v>AI-Based Traffic Management System</v>
       </c>
       <c r="C3" t="str">
         <v>Aarav Khadka, Binita Shrestha, Chandra Thapa</v>
@@ -448,11 +460,40 @@
       </c>
       <c r="E3" t="str">
         <v>2081</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Dr. Ram Acharya</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Prof. Hari Bhandari</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TeamBeta</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Smart Agriculture Monitoring Platform</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Dipesh Poudel, Ekta Rai, Firoj Khan</v>
+      </c>
+      <c r="D4" t="str">
+        <v>078BCT004, 078BEI001, 078BEI002</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2081</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Prof. Sita Sharma</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Dr. Sagar Ojha</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: batch auto-detection from roll number, fix templates, add template download routes, auto-fill startDate
</commit_message>
<xml_diff>
--- a/backend/excel-templates/bachelor_upload_template.xlsx
+++ b/backend/excel-templates/bachelor_upload_template.xlsx
@@ -397,7 +397,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G3"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="25.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="7" max="7" width="25.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,19 +416,19 @@
         <v>Project Title</v>
       </c>
       <c r="C1" t="str">
-        <v>Member Names</v>
+        <v>Members</v>
       </c>
       <c r="D1" t="str">
         <v>Roll Numbers</v>
       </c>
       <c r="E1" t="str">
-        <v>Academic Year</v>
+        <v>Batch</v>
       </c>
       <c r="F1" t="str">
         <v>Supervisor</v>
       </c>
       <c r="G1" t="str">
-        <v>Examiner</v>
+        <v>External Examiner</v>
       </c>
     </row>
     <row r="2">
@@ -459,41 +468,18 @@
         <v>078BCT001, 078BCT002, 078BCT003</v>
       </c>
       <c r="E3" t="str">
-        <v>2081</v>
+        <v>078</v>
       </c>
       <c r="F3" t="str">
         <v>Dr. Ram Acharya</v>
       </c>
       <c r="G3" t="str">
         <v>Prof. Hari Bhandari</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>TeamBeta</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Smart Agriculture Monitoring Platform</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Dipesh Poudel, Ekta Rai, Firoj Khan</v>
-      </c>
-      <c r="D4" t="str">
-        <v>078BCT004, 078BEI001, 078BEI002</v>
-      </c>
-      <c r="E4" t="str">
-        <v>2081</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Prof. Sita Sharma</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Dr. Sagar Ojha</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: evaluation system fixes, UI improvements, professional README
</commit_message>
<xml_diff>
--- a/backend/excel-templates/bachelor_upload_template.xlsx
+++ b/backend/excel-templates/bachelor_upload_template.xlsx
@@ -397,16 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="25.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="25.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:G4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -477,9 +468,32 @@
         <v>Prof. Hari Bhandari</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TeamBeta</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Smart Agriculture Monitoring Platform</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Dipesh Poudel, Ekta Rai, Firoj Khan</v>
+      </c>
+      <c r="D4" t="str">
+        <v>078BCT004, 078BCT005, 078BCT006</v>
+      </c>
+      <c r="E4" t="str">
+        <v>078</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Prof. Sita Sharma</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Dr. Sagar Ojha</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: enhance bachelor and master project workflows with cluster support, member editing, and response matrix fixes
</commit_message>
<xml_diff>
--- a/backend/excel-templates/bachelor_upload_template.xlsx
+++ b/backend/excel-templates/bachelor_upload_template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -416,9 +416,12 @@
         <v>Batch</v>
       </c>
       <c r="F1" t="str">
+        <v>Cluster</v>
+      </c>
+      <c r="G1" t="str">
         <v>Supervisor</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>External Examiner</v>
       </c>
     </row>
@@ -442,6 +445,9 @@
         <v/>
       </c>
       <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
         <v/>
       </c>
     </row>
@@ -462,9 +468,12 @@
         <v>078</v>
       </c>
       <c r="F3" t="str">
+        <v>AIML</v>
+      </c>
+      <c r="G3" t="str">
         <v>Dr. Ram Acharya</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>Prof. Hari Bhandari</v>
       </c>
     </row>
@@ -485,15 +494,18 @@
         <v>078</v>
       </c>
       <c r="F4" t="str">
+        <v>EDMES</v>
+      </c>
+      <c r="G4" t="str">
         <v>Prof. Sita Sharma</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>Dr. Sagar Ojha</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>